<commit_message>
Created github repo of slide drilling fixture based on the CAD template
</commit_message>
<xml_diff>
--- a/bom/bill of materials.xlsx
+++ b/bom/bill of materials.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rkiselev\Documents\dev\CAD-template\bom\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rkiselev\Documents\dev\CAD-indexed-slide-drilling-fixture\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A4A80D2-54B3-4DA7-9802-AD74E7088A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB933B9A-DE38-42FA-92B1-466198A1F7D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-4470" windowWidth="16440" windowHeight="28320" xr2:uid="{5E7C3FFB-AD92-4196-811B-21E5F425FF14}"/>
+    <workbookView xWindow="9075" yWindow="2025" windowWidth="32190" windowHeight="17700" xr2:uid="{5E7C3FFB-AD92-4196-811B-21E5F425FF14}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,17 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="65">
   <si>
     <t>Bill of materials</t>
   </si>
   <si>
-    <t>Raw aluminum</t>
-  </si>
-  <si>
-    <t>9246K524</t>
-  </si>
-  <si>
     <t>Vendor</t>
   </si>
   <si>
@@ -56,12 +50,6 @@
     <t>Formlabs</t>
   </si>
   <si>
-    <t>91698A202</t>
-  </si>
-  <si>
-    <t>M2x6 flat head screw</t>
-  </si>
-  <si>
     <t>Raw materials</t>
   </si>
   <si>
@@ -101,49 +89,148 @@
     <t>Material</t>
   </si>
   <si>
-    <t>6061-T6511 Al</t>
-  </si>
-  <si>
-    <t>Phillips Flat Head Screws, M2 x 0.4 mm, 6 mm Long</t>
-  </si>
-  <si>
-    <t>Multipurpose 6061-T6511 Aluminum, 5/8" Thick, 6" x 12"</t>
-  </si>
-  <si>
-    <t>pTIRF custom slide holder, v0.4.1</t>
-  </si>
-  <si>
     <t>Total</t>
   </si>
   <si>
     <t>3D printed parts (Formlabs Form 4)</t>
   </si>
   <si>
-    <t>CNC milled parts (HAAS VF-1)</t>
-  </si>
-  <si>
     <t>Pkg qty</t>
   </si>
   <si>
     <t>Mult.</t>
   </si>
   <si>
-    <t>Black Resin V5</t>
-  </si>
-  <si>
-    <t>RS-C2-GPBK-05</t>
-  </si>
-  <si>
-    <t>Black resin</t>
-  </si>
-  <si>
-    <t>Black Resin V5 (Form 4) 1 L</t>
-  </si>
-  <si>
-    <t>Gear</t>
-  </si>
-  <si>
-    <t>Frame</t>
+    <t>pTIRF indexed slide drilling fixture v1.0.0</t>
+  </si>
+  <si>
+    <t>302 Stainless Steel Compression Springs 0.75" Long, 0.18" OD, 0.148" ID</t>
+  </si>
+  <si>
+    <t>Compression springs</t>
+  </si>
+  <si>
+    <t>9435K22</t>
+  </si>
+  <si>
+    <t>Guide</t>
+  </si>
+  <si>
+    <t>Thorlabs</t>
+  </si>
+  <si>
+    <t>BA1L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BA1L - Mounting Base, 1" x 4.5" x 3/8" </t>
+  </si>
+  <si>
+    <t>Kinematic positioner</t>
+  </si>
+  <si>
+    <t>KL03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spring-Loaded Plunger, 0.85" (21.6 mm) Long Slot </t>
+  </si>
+  <si>
+    <t>Aluminum breadboard</t>
+  </si>
+  <si>
+    <t>MSB6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6" x  6" x 3/8" Mini-Series Aluminum Breadboard, 8-32 and 1/4"-20 Taps </t>
+  </si>
+  <si>
+    <t>6" x 12" x 1/16" cast acrylic sheet</t>
+  </si>
+  <si>
+    <t>6" x 12" x 3/32" cast acrylic sheet</t>
+  </si>
+  <si>
+    <t>6" x 12" x 7/32" cast acrylic sheet</t>
+  </si>
+  <si>
+    <t>6" x 12" x 1/4" cast acrylic sheet</t>
+  </si>
+  <si>
+    <t>8560K178</t>
+  </si>
+  <si>
+    <t>8560K188</t>
+  </si>
+  <si>
+    <t>8560K179</t>
+  </si>
+  <si>
+    <t>8560K359</t>
+  </si>
+  <si>
+    <t>RS-C2-TO20-11</t>
+  </si>
+  <si>
+    <t>Tough 2000 Resin (Form 4) 1 L</t>
+  </si>
+  <si>
+    <t>Tough 2000 resin</t>
+  </si>
+  <si>
+    <t>Slide drilling fixture base</t>
+  </si>
+  <si>
+    <t>Slide drilling fixture top</t>
+  </si>
+  <si>
+    <t>Slide drilling plunger</t>
+  </si>
+  <si>
+    <t>1/16" acrylic</t>
+  </si>
+  <si>
+    <t>1/16" (1.6mm) acrylic glass</t>
+  </si>
+  <si>
+    <t>3/32" (2.4mm) acrylic glass</t>
+  </si>
+  <si>
+    <t>7/32" (5.6mm) acrylic glass</t>
+  </si>
+  <si>
+    <t>1/4" (6.4mm) acrylic glass</t>
+  </si>
+  <si>
+    <t>Slide drilling fixture bottom</t>
+  </si>
+  <si>
+    <t>3/32" acrylic</t>
+  </si>
+  <si>
+    <t>Slide drilling fixture pedestal</t>
+  </si>
+  <si>
+    <t>Slide drilling fixture plunger</t>
+  </si>
+  <si>
+    <t>7/32" acrylic</t>
+  </si>
+  <si>
+    <t>1/4" acrylic</t>
+  </si>
+  <si>
+    <t>a) laser cut and fused with dichloromethane, or</t>
+  </si>
+  <si>
+    <t>b) 3D printed and glued with superglue</t>
+  </si>
+  <si>
+    <t>NOTE</t>
+  </si>
+  <si>
+    <t>The slide drilling fixture can be either</t>
+  </si>
+  <si>
+    <t>Laser cut parts (Universal laser VLS2.30)</t>
   </si>
 </sst>
 </file>
@@ -154,7 +241,7 @@
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,6 +288,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -210,7 +303,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -251,6 +344,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -263,7 +367,7 @@
   <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -271,13 +375,13 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="2" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="2" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -629,19 +733,19 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.5703125" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.42578125" customWidth="1"/>
     <col min="6" max="6" width="9.42578125" customWidth="1"/>
     <col min="7" max="7" width="7.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="5.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.7109375" customWidth="1"/>
-    <col min="10" max="10" width="55.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="64.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -660,12 +764,12 @@
     </row>
     <row r="2" spans="1:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="18" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="17" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B4" s="17"/>
       <c r="C4" s="17"/>
@@ -680,39 +784,39 @@
     <row r="5" spans="1:10" ht="9" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:10" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="15" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
@@ -729,74 +833,140 @@
         <v>1</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="E8" s="5">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F8" s="8">
-        <v>9.7200000000000006</v>
+        <v>5.76</v>
       </c>
       <c r="G8" s="11">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="H8" s="12">
         <f>E8/G8</f>
-        <v>0.12</v>
+        <v>0.4</v>
       </c>
       <c r="I8" s="9">
         <f>F8*H8</f>
-        <v>1.1664000000000001</v>
+        <v>2.3039999999999998</v>
       </c>
       <c r="J8" s="5" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="5"/>
+      <c r="A9" s="5">
+        <v>2</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="5">
+        <v>1</v>
+      </c>
+      <c r="F9" s="8">
+        <v>14.53</v>
+      </c>
+      <c r="G9" s="11">
+        <v>1</v>
+      </c>
+      <c r="H9" s="12">
+        <f t="shared" ref="H9:H10" si="0">E9/G9</f>
+        <v>1</v>
+      </c>
+      <c r="I9" s="9">
+        <f t="shared" ref="I9:I10" si="1">F9*H9</f>
+        <v>14.53</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="5"/>
+      <c r="A10" s="5">
+        <v>3</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="5">
+        <v>1</v>
+      </c>
+      <c r="F10" s="8">
+        <v>7.76</v>
+      </c>
+      <c r="G10" s="11">
+        <v>1</v>
+      </c>
+      <c r="H10" s="12">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="I10" s="9">
+        <f t="shared" si="1"/>
+        <v>7.76</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="5"/>
+      <c r="A11" s="5">
+        <v>4</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="5">
+        <v>1</v>
+      </c>
+      <c r="F11" s="8">
+        <v>8.76</v>
+      </c>
+      <c r="G11" s="11">
+        <v>2</v>
+      </c>
+      <c r="H11" s="12">
+        <f t="shared" ref="H11" si="2">E11/G11</f>
+        <v>0.5</v>
+      </c>
+      <c r="I11" s="9">
+        <f t="shared" ref="I11" si="3">F11*H11</f>
+        <v>4.38</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B12" s="15"/>
       <c r="C12" s="15"/>
@@ -813,19 +983,19 @@
         <v>1</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="E13" s="5">
         <v>1</v>
       </c>
       <c r="F13" s="8">
-        <v>49.95</v>
+        <v>3.44</v>
       </c>
       <c r="G13" s="11">
         <v>1</v>
@@ -836,10 +1006,10 @@
       </c>
       <c r="I13" s="9">
         <f>F13*H13</f>
-        <v>49.95</v>
+        <v>3.44</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -847,175 +1017,367 @@
         <v>2</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="5">
+        <v>1</v>
+      </c>
+      <c r="F14" s="8">
+        <v>3.65</v>
+      </c>
+      <c r="G14" s="11">
+        <v>1</v>
+      </c>
+      <c r="H14" s="12">
+        <f t="shared" ref="H14:H16" si="4">E14/G14</f>
+        <v>1</v>
+      </c>
+      <c r="I14" s="9">
+        <f t="shared" ref="I14:I16" si="5">F14*H14</f>
+        <v>3.65</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="5">
+        <v>3</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" s="5">
+        <v>1</v>
+      </c>
+      <c r="F15" s="8">
+        <v>9.92</v>
+      </c>
+      <c r="G15" s="11">
+        <v>1</v>
+      </c>
+      <c r="H15" s="12">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="I15" s="9">
+        <f t="shared" si="5"/>
+        <v>9.92</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="5">
+        <v>4</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" s="5">
+        <v>1</v>
+      </c>
+      <c r="F16" s="8">
+        <v>13.96</v>
+      </c>
+      <c r="G16" s="11">
+        <v>1</v>
+      </c>
+      <c r="H16" s="12">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="I16" s="9">
+        <f t="shared" si="5"/>
+        <v>13.96</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="5">
         <v>5</v>
       </c>
-      <c r="D14" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="E14" s="13">
-        <v>73</v>
-      </c>
-      <c r="F14" s="14">
-        <v>79</v>
-      </c>
-      <c r="G14" s="11">
+      <c r="B17" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" s="5">
+        <v>50</v>
+      </c>
+      <c r="F17" s="13">
+        <v>149</v>
+      </c>
+      <c r="G17" s="11">
         <v>1000</v>
       </c>
-      <c r="H14" s="12">
-        <f>E14/G14</f>
-        <v>7.2999999999999995E-2</v>
-      </c>
-      <c r="I14" s="9">
-        <f>F14*H14</f>
-        <v>5.7669999999999995</v>
-      </c>
-      <c r="J14" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="D15" s="1"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="I15" s="9">
-        <f>SUM(I8:I14)</f>
-        <v>56.883400000000009</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="17"/>
-    </row>
-    <row r="17" spans="1:9" ht="6" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>20</v>
-      </c>
+      <c r="H17" s="12">
+        <f>E17/G17</f>
+        <v>0.05</v>
+      </c>
+      <c r="I17" s="9">
+        <f>F17*H17</f>
+        <v>7.45</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="14"/>
+      <c r="D18" s="1"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
-      <c r="I18" s="3"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="I19" s="3"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="5">
-        <v>1</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C20" s="5">
-        <v>1</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="I20" s="3"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
+      <c r="H18" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I18" s="9">
+        <f>SUM(I8:I17)</f>
+        <v>67.394000000000005</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="18" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17"/>
+    </row>
+    <row r="20" spans="1:10" ht="6" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="I21" s="3"/>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A22" s="5">
-        <v>1</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C22" s="5">
-        <v>1</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="F22" s="2"/>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="F22" s="2" t="s">
+        <v>62</v>
+      </c>
       <c r="G22" s="2"/>
       <c r="I22" s="3"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="5">
+        <v>1</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="5">
+        <v>1</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>63</v>
+      </c>
       <c r="I23" s="3"/>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="5">
+        <v>2</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" s="5">
+        <v>1</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="I24" s="3"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A25" s="5"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="5">
+        <v>3</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C25" s="5">
+        <v>1</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G25" s="2"/>
+      <c r="I25" s="3"/>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="5">
+        <v>4</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" s="5">
+        <v>2</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="I26" s="3"/>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
+        <v>5</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" s="5">
+        <v>1</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G27" s="2"/>
+      <c r="I27" s="3"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="G28" s="2"/>
+      <c r="I28" s="3"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>1</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C29" s="5">
+        <v>1</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="I29" s="3"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="5">
+        <v>2</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C30" s="5">
+        <v>1</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="I30" s="3"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="5">
+        <v>3</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C31" s="5">
+        <v>2</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="I31" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A28:D28"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A4:J4"/>
-    <mergeCell ref="A16:J16"/>
+    <mergeCell ref="A19:J19"/>
     <mergeCell ref="A7:J7"/>
     <mergeCell ref="A12:J12"/>
   </mergeCells>
+  <phoneticPr fontId="6" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D13" r:id="rId1" xr:uid="{A92ED648-F042-4DB1-BDA2-ACF6A8003DF9}"/>
     <hyperlink ref="D8" r:id="rId2" xr:uid="{2B374A49-030C-4787-B652-5E0666B02CFB}"/>
-    <hyperlink ref="D14" r:id="rId3" xr:uid="{F14FA5A5-4C71-4F6A-AACF-1FB846D53597}"/>
+    <hyperlink ref="D9" r:id="rId3" xr:uid="{803F430D-31E2-44DF-8B90-F0730A94B8DA}"/>
+    <hyperlink ref="D10" r:id="rId4" xr:uid="{B3412580-B8ED-4458-9C65-6C4549FA2886}"/>
+    <hyperlink ref="D11" r:id="rId5" xr:uid="{EFFC1B77-F917-4395-A290-70557A2E4742}"/>
+    <hyperlink ref="D14" r:id="rId6" xr:uid="{4433A976-CC2A-4FF8-956F-859A6CC82D24}"/>
+    <hyperlink ref="D15" r:id="rId7" xr:uid="{22AC35E2-523A-4BD8-87CC-33AD2C07F085}"/>
+    <hyperlink ref="D16" r:id="rId8" xr:uid="{E20A9D33-39B4-4536-83DF-B89316E9B460}"/>
+    <hyperlink ref="D17" r:id="rId9" xr:uid="{7D7F4773-9466-494B-A066-4E4A4938398E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="87" orientation="landscape" r:id="rId4"/>
+  <pageSetup scale="87" orientation="landscape" r:id="rId10"/>
 </worksheet>
 </file>
</xml_diff>